<commit_message>
style: enhance web UI professionalism, transition Crosswalk color to Green, display all boundary curves simultaneously, and format Excel chart gridlines & units
</commit_message>
<xml_diff>
--- a/nchrp_562_calculations.xlsx
+++ b/nchrp_562_calculations.xlsx
@@ -241,13 +241,13 @@
       <font>
         <name val="Segoe UI"/>
         <b val="1"/>
-        <color rgb="000070C0"/>
+        <color rgb="00375623"/>
         <sz val="10"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00DDEBF7"/>
-          <bgColor rgb="00DDEBF7"/>
+          <fgColor rgb="00E2EFDA"/>
+          <bgColor rgb="00E2EFDA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -405,7 +405,7 @@
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
-                <a:srgbClr val="1565C0"/>
+                <a:srgbClr val="2E7D32"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -566,6 +566,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="20"/>
+        <majorUnit val="300"/>
       </valAx>
       <valAx>
         <axId val="20"/>
@@ -594,6 +595,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <majorUnit val="100"/>
       </valAx>
     </plotArea>
     <legend>
@@ -798,6 +800,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="20"/>
+        <majorUnit val="300"/>
       </valAx>
       <valAx>
         <axId val="20"/>
@@ -826,6 +829,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <majorUnit val="100"/>
       </valAx>
     </plotArea>
     <legend>

</xml_diff>

<commit_message>
Cap signal warrant curve calculations at parabola vertices to prevent upward curling and ensure correct warrant evaluation at high volumes
</commit_message>
<xml_diff>
--- a/nchrp_562_calculations.xlsx
+++ b/nchrp_562_calculations.xlsx
@@ -1580,7 +1580,7 @@
         </is>
       </c>
       <c r="C18" s="13">
-        <f>(0.00021 * C17^2 - 0.74072 * C17 + 734.125)/0.75</f>
+        <f>(0.00021 * MIN(C17, 1764)^2 - 0.74072 * MIN(C17, 1764) + 734.125)/0.75</f>
         <v/>
       </c>
     </row>
@@ -2324,7 +2324,7 @@
         </is>
       </c>
       <c r="C18" s="13">
-        <f>(0.00035 * C17^2 - 0.80083 * C17 + 529.197)/0.75</f>
+        <f>(0.00035 * MIN(C17, 1144)^2 - 0.80083 * MIN(C17, 1144) + 529.197)/0.75</f>
         <v/>
       </c>
     </row>

</xml_diff>